<commit_message>
Actualizar S27: nueva estructura datos + YoY mermas en Riesgos
- Base exactitud: ahora una sola hoja (Base Cuentas, S01-S27)
- Stock: nueva hoja/columnas (Stock disp, Bloqueado, XLIB)
- Quiebres: comentarios hasta S27 (404 comentarios)
- Nuevo KPI: Venta Sell IN YoY YTD (2026 vs 2025 acumulado)
- Tabla Riesgos: nueva columna %YoY por SKU vs mismo período 2025
- Datos: 329.8t quebrado S27, 188 críticos, 134 alertas, -10.5% YoY

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fpDzYDGDx6YjRFmdKtXpg
</commit_message>
<xml_diff>
--- a/exactitud-semanal/Principales_Productos_con_Quiebres.xlsx
+++ b/exactitud-semanal/Principales_Productos_con_Quiebres.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9303"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="2160" windowHeight="1050"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="2160" windowHeight="1185"/>
   </bookViews>
   <sheets>
     <sheet name="Principales Productos con Quieb" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1348" uniqueCount="584">
   <si>
     <t xml:space="preserve">Semana </t>
   </si>
@@ -1536,6 +1536,156 @@
   </si>
   <si>
     <t>Stock XLIB</t>
+  </si>
+  <si>
+    <t>QUESO LAS PARCELAS LAMIN 16X350GR</t>
+  </si>
+  <si>
+    <t>QUESO LPV LAM S/BORDE 12X470G</t>
+  </si>
+  <si>
+    <t>Bloqueo comercial</t>
+  </si>
+  <si>
+    <t>MARGARINA SUREÑA MIX 6X900GR</t>
+  </si>
+  <si>
+    <t>Laminadora fuera de servicio</t>
+  </si>
+  <si>
+    <t>ACEITE CHEF EXTRAVIRGEN 6X1LT</t>
+  </si>
+  <si>
+    <t>MERMELADA WATTS FRAMBUESA FRASCO 10X500G</t>
+  </si>
+  <si>
+    <t>MERMELADA WATTS S/A FBSA SACHET 24X200GR</t>
+  </si>
+  <si>
+    <t>POROTOS BLANCOS SIN SAL WASIL 16X340GR</t>
+  </si>
+  <si>
+    <t>Producto descontinuado</t>
+  </si>
+  <si>
+    <t>Quiebre por empalme se producirá hasta agotar ME</t>
+  </si>
+  <si>
+    <t>LECHE POLVO CALO ENTERA INST 20X850GR</t>
+  </si>
+  <si>
+    <t>Mantención de la linea</t>
+  </si>
+  <si>
+    <t>QUESO LAS PARCELAS LAM 4X2,5KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">atraso en la liberacion </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desvio de demanda / duplico su fcst </t>
+  </si>
+  <si>
+    <t>Walmart triplico su fcst / Libera 8 tons</t>
+  </si>
+  <si>
+    <t>YOGURT YOGU YOGU MORA BOT 6X900GR</t>
+  </si>
+  <si>
+    <t>desvio de demanda - empalme / libera 10 tons</t>
+  </si>
+  <si>
+    <t>JUGO FRESCO WATTS NJA ZANAHORIA 6X1,6LT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">atraso en concentrado / stock en transito </t>
+  </si>
+  <si>
+    <t xml:space="preserve">desvio de demanda - empalme </t>
+  </si>
+  <si>
+    <t>JUGO FRESCO WATTS NARANJA-PIÑA 6X1,6LT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">empalme - stock en transito </t>
+  </si>
+  <si>
+    <t>NECTAR WATTS MANZANA 5X10X115ML</t>
+  </si>
+  <si>
+    <t>Retraso de Linea</t>
+  </si>
+  <si>
+    <t>Retraso en llegada de proteina</t>
+  </si>
+  <si>
+    <t>Ya cumplió su SOP de Junio</t>
+  </si>
+  <si>
+    <t>Bloqueo marketing</t>
+  </si>
+  <si>
+    <t>MANGO EN TROZOS WASIL 16X500G</t>
+  </si>
+  <si>
+    <t>Llegadas intermitentes de ME (tapas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">falla de maquina / empalme </t>
+  </si>
+  <si>
+    <t xml:space="preserve">falla de linea </t>
+  </si>
+  <si>
+    <t>LECHE POLVO LONCO SEMIDESCREMADA10X760GR</t>
+  </si>
+  <si>
+    <t>A la espera de ME</t>
+  </si>
+  <si>
+    <t>ACEITE MAZOLA CANOLA 12X1LT</t>
+  </si>
+  <si>
+    <t>% de aceptación Santa Isabel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuertes compras por recuperacion / empalme </t>
+  </si>
+  <si>
+    <t>FRUGO MARACUYA 6X1,6LT</t>
+  </si>
+  <si>
+    <t>Desvio de demada / 6 tons prox liberacion</t>
+  </si>
+  <si>
+    <t>Fuertes compras por recuperacion / 7 tons en la siguiente liberacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empalme / 5 tons dispobibles </t>
+  </si>
+  <si>
+    <t>YOG LONCO PROTEIN NAT S/E BALDE 6X800GR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desvio de demanda / 5 tons prox semana </t>
+  </si>
+  <si>
+    <t>ACEITE CRISTAL VEGETAL 12X900ML</t>
+  </si>
+  <si>
+    <t>% VU</t>
+  </si>
+  <si>
+    <t>ACEITE CHEF MARAVILLA 12X1LT</t>
+  </si>
+  <si>
+    <t>Falta MP, Recupera SEM 29</t>
+  </si>
+  <si>
+    <t>Se priorizó otros sku de Maquina Prisma</t>
+  </si>
+  <si>
+    <t>MANJAR LONCOLECHE BOLSA 10X920GR</t>
   </si>
   <si>
     <t>PASTA CHOCLO 12X500GR</t>
@@ -1792,7 +1942,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1804,26 +1953,23 @@
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -2405,10 +2551,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2734,7 +2880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L367"/>
+  <dimension ref="A1:L454"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="22.85546875" customWidth="1"/>
@@ -8370,6 +8516,9 @@
       <c r="D294" s="5">
         <v>1031</v>
       </c>
+      <c r="E294" t="s">
+        <v>147</v>
+      </c>
     </row>
     <row r="295" spans="1:6">
       <c r="A295">
@@ -9823,6 +9972,1692 @@
         <v>46183</v>
       </c>
       <c r="G367" s="54"/>
+    </row>
+    <row r="368" spans="1:7">
+      <c r="A368">
+        <v>202624</v>
+      </c>
+      <c r="B368" s="56">
+        <v>30001862</v>
+      </c>
+      <c r="C368" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D368" s="5">
+        <v>22.518000000000001</v>
+      </c>
+      <c r="E368" t="s">
+        <v>225</v>
+      </c>
+      <c r="F368" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="369" spans="1:6">
+      <c r="A369">
+        <v>202624</v>
+      </c>
+      <c r="B369" s="56">
+        <v>30001689</v>
+      </c>
+      <c r="C369" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D369" s="5">
+        <v>7.2488000000000001</v>
+      </c>
+      <c r="E369" t="s">
+        <v>225</v>
+      </c>
+      <c r="F369" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="370" spans="1:6">
+      <c r="A370">
+        <v>202624</v>
+      </c>
+      <c r="B370" s="56">
+        <v>30000560</v>
+      </c>
+      <c r="C370" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="D370" s="5">
+        <v>5.1016000000000004</v>
+      </c>
+      <c r="E370" t="s">
+        <v>225</v>
+      </c>
+      <c r="F370" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="371" spans="1:6">
+      <c r="A371">
+        <v>202624</v>
+      </c>
+      <c r="B371" s="56">
+        <v>30001400</v>
+      </c>
+      <c r="C371" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="D371" s="5">
+        <v>4.8221999999999996</v>
+      </c>
+      <c r="E371" t="s">
+        <v>502</v>
+      </c>
+      <c r="F371" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="372" spans="1:6">
+      <c r="A372">
+        <v>202624</v>
+      </c>
+      <c r="B372" s="56">
+        <v>30001774</v>
+      </c>
+      <c r="C372" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D372" s="5">
+        <v>4.4400000000000004</v>
+      </c>
+      <c r="E372" t="s">
+        <v>225</v>
+      </c>
+      <c r="F372" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="373" spans="1:6">
+      <c r="A373">
+        <v>202624</v>
+      </c>
+      <c r="B373" s="56">
+        <v>30001935</v>
+      </c>
+      <c r="C373" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="D373" s="5">
+        <v>3.70608</v>
+      </c>
+      <c r="E373" t="s">
+        <v>225</v>
+      </c>
+      <c r="F373" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="374" spans="1:6">
+      <c r="A374">
+        <v>202624</v>
+      </c>
+      <c r="B374" s="56">
+        <v>30002253</v>
+      </c>
+      <c r="C374" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D374" s="5">
+        <v>3.1320000000000001</v>
+      </c>
+      <c r="E374" t="s">
+        <v>225</v>
+      </c>
+      <c r="F374" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="375" spans="1:6">
+      <c r="A375">
+        <v>202624</v>
+      </c>
+      <c r="B375" s="56">
+        <v>30000466</v>
+      </c>
+      <c r="C375" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D375" s="5">
+        <v>2.9279999999999999</v>
+      </c>
+      <c r="E375" t="s">
+        <v>504</v>
+      </c>
+      <c r="F375" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="376" spans="1:6">
+      <c r="A376">
+        <v>202624</v>
+      </c>
+      <c r="B376" s="56">
+        <v>30000194</v>
+      </c>
+      <c r="C376" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D376" s="5">
+        <v>6.2729999999999997</v>
+      </c>
+      <c r="E376" t="s">
+        <v>484</v>
+      </c>
+      <c r="F376" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="377" spans="1:6">
+      <c r="A377">
+        <v>202624</v>
+      </c>
+      <c r="B377" s="56">
+        <v>30001362</v>
+      </c>
+      <c r="C377" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="D377" s="5">
+        <v>3.9412799999999999</v>
+      </c>
+      <c r="E377" t="s">
+        <v>477</v>
+      </c>
+      <c r="F377" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="378" spans="1:6">
+      <c r="A378">
+        <v>202624</v>
+      </c>
+      <c r="B378" s="56">
+        <v>30001142</v>
+      </c>
+      <c r="C378" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D378" s="5">
+        <v>2.77</v>
+      </c>
+      <c r="E378" t="s">
+        <v>484</v>
+      </c>
+      <c r="F378" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="379" spans="1:6">
+      <c r="A379">
+        <v>202624</v>
+      </c>
+      <c r="B379" s="56">
+        <v>30002113</v>
+      </c>
+      <c r="C379" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D379" s="5">
+        <v>2.3050000000000002</v>
+      </c>
+      <c r="E379" t="s">
+        <v>484</v>
+      </c>
+      <c r="F379" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="380" spans="1:6">
+      <c r="A380">
+        <v>202624</v>
+      </c>
+      <c r="B380" s="56">
+        <v>30000179</v>
+      </c>
+      <c r="C380" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="D380" s="5">
+        <v>2.04</v>
+      </c>
+      <c r="E380" t="s">
+        <v>486</v>
+      </c>
+      <c r="F380" s="54">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="381" spans="1:6">
+      <c r="A381">
+        <v>202624</v>
+      </c>
+      <c r="B381" s="56">
+        <v>30002114</v>
+      </c>
+      <c r="C381" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D381" s="5">
+        <v>1.2749999999999999</v>
+      </c>
+      <c r="E381" t="s">
+        <v>484</v>
+      </c>
+      <c r="F381" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="382" spans="1:6">
+      <c r="A382">
+        <v>202624</v>
+      </c>
+      <c r="B382" s="56">
+        <v>30001365</v>
+      </c>
+      <c r="C382" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="D382" s="5">
+        <v>1.2430000000000001</v>
+      </c>
+      <c r="E382" t="s">
+        <v>477</v>
+      </c>
+      <c r="F382" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="383" spans="1:6">
+      <c r="A383">
+        <v>202624</v>
+      </c>
+      <c r="B383" s="56">
+        <v>30001741</v>
+      </c>
+      <c r="C383" s="5" t="s">
+        <v>508</v>
+      </c>
+      <c r="D383" s="5">
+        <v>1.1152</v>
+      </c>
+      <c r="E383" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="384" spans="1:6">
+      <c r="A384">
+        <v>202624</v>
+      </c>
+      <c r="B384" s="56">
+        <v>30001411</v>
+      </c>
+      <c r="C384" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="D384" s="5">
+        <v>15.282</v>
+      </c>
+      <c r="E384" t="s">
+        <v>510</v>
+      </c>
+      <c r="F384" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="385" spans="1:6">
+      <c r="A385">
+        <v>202624</v>
+      </c>
+      <c r="B385" s="56">
+        <v>30001409</v>
+      </c>
+      <c r="C385" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="D385" s="5">
+        <v>12.308</v>
+      </c>
+      <c r="E385" t="s">
+        <v>421</v>
+      </c>
+      <c r="F385" s="54">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="386" spans="1:6">
+      <c r="A386">
+        <v>202624</v>
+      </c>
+      <c r="B386" s="56">
+        <v>30001405</v>
+      </c>
+      <c r="C386" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="D386" s="5">
+        <v>7.9379999999999997</v>
+      </c>
+      <c r="E386" t="s">
+        <v>486</v>
+      </c>
+      <c r="F386" s="54">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="387" spans="1:6">
+      <c r="A387">
+        <v>202624</v>
+      </c>
+      <c r="B387" s="56">
+        <v>30001404</v>
+      </c>
+      <c r="C387" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D387" s="5">
+        <v>7.569</v>
+      </c>
+      <c r="E387" t="s">
+        <v>486</v>
+      </c>
+      <c r="F387" s="54">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="388" spans="1:6">
+      <c r="A388">
+        <v>202624</v>
+      </c>
+      <c r="B388" s="56">
+        <v>30001423</v>
+      </c>
+      <c r="C388" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="D388" s="5">
+        <v>7.4924999999999997</v>
+      </c>
+      <c r="E388" t="s">
+        <v>486</v>
+      </c>
+      <c r="F388" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="389" spans="1:6">
+      <c r="A389">
+        <v>202624</v>
+      </c>
+      <c r="B389" s="56">
+        <v>30001376</v>
+      </c>
+      <c r="C389" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D389" s="5">
+        <v>6.5114999999999998</v>
+      </c>
+      <c r="E389" t="s">
+        <v>486</v>
+      </c>
+      <c r="F389" s="54">
+        <v>46215</v>
+      </c>
+    </row>
+    <row r="390" spans="1:6">
+      <c r="A390">
+        <v>202624</v>
+      </c>
+      <c r="B390" s="56">
+        <v>30001980</v>
+      </c>
+      <c r="C390" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D390" s="5">
+        <v>5.1974999999999998</v>
+      </c>
+      <c r="E390" t="s">
+        <v>486</v>
+      </c>
+      <c r="F390" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="391" spans="1:6">
+      <c r="A391">
+        <v>202624</v>
+      </c>
+      <c r="B391" s="56">
+        <v>30000522</v>
+      </c>
+      <c r="C391" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="D391" s="5">
+        <v>4.7160000000000002</v>
+      </c>
+      <c r="E391" t="s">
+        <v>512</v>
+      </c>
+      <c r="F391" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="392" spans="1:6">
+      <c r="A392">
+        <v>202625</v>
+      </c>
+      <c r="B392" s="56">
+        <v>30001815</v>
+      </c>
+      <c r="C392" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="D392" s="5">
+        <v>8.39</v>
+      </c>
+      <c r="E392" t="s">
+        <v>514</v>
+      </c>
+      <c r="F392" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="393" spans="1:6">
+      <c r="A393">
+        <v>202625</v>
+      </c>
+      <c r="B393" s="56">
+        <v>30001689</v>
+      </c>
+      <c r="C393" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D393" s="5">
+        <v>7.4568000000000003</v>
+      </c>
+      <c r="E393" t="s">
+        <v>225</v>
+      </c>
+      <c r="F393" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="394" spans="1:6">
+      <c r="A394">
+        <v>202625</v>
+      </c>
+      <c r="B394" s="56">
+        <v>30000560</v>
+      </c>
+      <c r="C394" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="D394" s="5">
+        <v>4.9168000000000003</v>
+      </c>
+      <c r="E394" t="s">
+        <v>515</v>
+      </c>
+      <c r="F394" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="395" spans="1:6">
+      <c r="A395">
+        <v>202625</v>
+      </c>
+      <c r="B395" s="56">
+        <v>30001773</v>
+      </c>
+      <c r="C395" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="D395" s="5">
+        <v>4.194</v>
+      </c>
+      <c r="E395" t="s">
+        <v>516</v>
+      </c>
+      <c r="F395" s="54">
+        <v>46201</v>
+      </c>
+    </row>
+    <row r="396" spans="1:6">
+      <c r="A396">
+        <v>202625</v>
+      </c>
+      <c r="B396" s="56">
+        <v>30001901</v>
+      </c>
+      <c r="C396" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D396" s="5">
+        <v>3.0131999999999999</v>
+      </c>
+      <c r="E396" t="s">
+        <v>518</v>
+      </c>
+      <c r="F396" s="54">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="397" spans="1:6">
+      <c r="A397">
+        <v>202625</v>
+      </c>
+      <c r="B397" s="56">
+        <v>30002135</v>
+      </c>
+      <c r="C397" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="D397" s="5">
+        <v>2.8512</v>
+      </c>
+      <c r="E397" t="s">
+        <v>520</v>
+      </c>
+      <c r="F397" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="398" spans="1:6">
+      <c r="A398">
+        <v>202625</v>
+      </c>
+      <c r="B398" s="56">
+        <v>30001862</v>
+      </c>
+      <c r="C398" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="D398" s="5">
+        <v>2.5920000000000001</v>
+      </c>
+      <c r="E398" t="s">
+        <v>521</v>
+      </c>
+      <c r="F398" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="399" spans="1:6">
+      <c r="A399">
+        <v>202625</v>
+      </c>
+      <c r="B399" s="56">
+        <v>30002134</v>
+      </c>
+      <c r="C399" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="D399" s="5">
+        <v>2.2848000000000002</v>
+      </c>
+      <c r="E399" t="s">
+        <v>523</v>
+      </c>
+      <c r="F399" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="400" spans="1:6">
+      <c r="A400">
+        <v>202625</v>
+      </c>
+      <c r="B400" s="56">
+        <v>30001939</v>
+      </c>
+      <c r="C400" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D400" s="5">
+        <v>2.0255999999999998</v>
+      </c>
+      <c r="E400" t="s">
+        <v>523</v>
+      </c>
+      <c r="F400" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="401" spans="1:6">
+      <c r="A401">
+        <v>202625</v>
+      </c>
+      <c r="B401" s="56">
+        <v>30000522</v>
+      </c>
+      <c r="C401" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="D401" s="5">
+        <v>41.448</v>
+      </c>
+      <c r="E401" t="s">
+        <v>512</v>
+      </c>
+      <c r="F401" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="402" spans="1:6">
+      <c r="A402">
+        <v>202625</v>
+      </c>
+      <c r="B402" s="56">
+        <v>30001409</v>
+      </c>
+      <c r="C402" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="D402" s="5">
+        <v>41.326999999999998</v>
+      </c>
+      <c r="E402" t="s">
+        <v>421</v>
+      </c>
+      <c r="F402" s="54">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="403" spans="1:6">
+      <c r="A403">
+        <v>202625</v>
+      </c>
+      <c r="B403" s="56">
+        <v>30002230</v>
+      </c>
+      <c r="C403" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="D403" s="5">
+        <v>11.292999999999999</v>
+      </c>
+      <c r="E403" t="s">
+        <v>525</v>
+      </c>
+      <c r="F403" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="404" spans="1:6">
+      <c r="A404">
+        <v>202625</v>
+      </c>
+      <c r="B404" s="56">
+        <v>30001376</v>
+      </c>
+      <c r="C404" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D404" s="5">
+        <v>9.5625</v>
+      </c>
+      <c r="E404" t="s">
+        <v>526</v>
+      </c>
+      <c r="F404" s="54">
+        <v>46215</v>
+      </c>
+    </row>
+    <row r="405" spans="1:6">
+      <c r="A405">
+        <v>202625</v>
+      </c>
+      <c r="B405" s="56">
+        <v>30001404</v>
+      </c>
+      <c r="C405" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D405" s="5">
+        <v>9.3330000000000002</v>
+      </c>
+      <c r="E405" t="s">
+        <v>255</v>
+      </c>
+      <c r="F405" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="406" spans="1:6">
+      <c r="A406">
+        <v>202625</v>
+      </c>
+      <c r="B406" s="56">
+        <v>30002228</v>
+      </c>
+      <c r="C406" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D406" s="5">
+        <v>7.9809999999999999</v>
+      </c>
+      <c r="E406" t="s">
+        <v>527</v>
+      </c>
+      <c r="F406" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="407" spans="1:6">
+      <c r="A407">
+        <v>202625</v>
+      </c>
+      <c r="B407" s="56">
+        <v>30001980</v>
+      </c>
+      <c r="C407" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D407" s="5">
+        <v>5.58</v>
+      </c>
+      <c r="E407" t="s">
+        <v>255</v>
+      </c>
+      <c r="F407" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="408" spans="1:6">
+      <c r="A408">
+        <v>202625</v>
+      </c>
+      <c r="B408" s="56">
+        <v>30000543</v>
+      </c>
+      <c r="C408" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="D408" s="5">
+        <v>4.2720000000000002</v>
+      </c>
+      <c r="E408" t="s">
+        <v>514</v>
+      </c>
+      <c r="F408" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="409" spans="1:6">
+      <c r="A409">
+        <v>202625</v>
+      </c>
+      <c r="B409" s="56">
+        <v>30001407</v>
+      </c>
+      <c r="C409" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="D409" s="5">
+        <v>4.2344999999999997</v>
+      </c>
+      <c r="E409" t="s">
+        <v>255</v>
+      </c>
+      <c r="F409" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="410" spans="1:6">
+      <c r="A410">
+        <v>202625</v>
+      </c>
+      <c r="B410" s="56">
+        <v>30000179</v>
+      </c>
+      <c r="C410" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="D410" s="5">
+        <v>7.0895999999999999</v>
+      </c>
+      <c r="E410" t="s">
+        <v>375</v>
+      </c>
+      <c r="F410" s="54">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="411" spans="1:6">
+      <c r="A411">
+        <v>202625</v>
+      </c>
+      <c r="B411" s="56">
+        <v>30001362</v>
+      </c>
+      <c r="C411" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="D411" s="5">
+        <v>4.8686400000000001</v>
+      </c>
+      <c r="E411" t="s">
+        <v>477</v>
+      </c>
+      <c r="F411" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="412" spans="1:6">
+      <c r="A412">
+        <v>202625</v>
+      </c>
+      <c r="B412" s="56">
+        <v>30001142</v>
+      </c>
+      <c r="C412" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D412" s="5">
+        <v>2.4849999999999999</v>
+      </c>
+      <c r="E412" t="s">
+        <v>484</v>
+      </c>
+      <c r="F412" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="413" spans="1:6">
+      <c r="A413">
+        <v>202625</v>
+      </c>
+      <c r="B413" s="56">
+        <v>30000194</v>
+      </c>
+      <c r="C413" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D413" s="5">
+        <v>1.641</v>
+      </c>
+      <c r="E413" t="s">
+        <v>528</v>
+      </c>
+      <c r="F413" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="414" spans="1:6">
+      <c r="A414">
+        <v>202625</v>
+      </c>
+      <c r="B414" s="56">
+        <v>30002138</v>
+      </c>
+      <c r="C414" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="D414" s="5">
+        <v>1.528</v>
+      </c>
+      <c r="E414" t="s">
+        <v>35</v>
+      </c>
+      <c r="F414" s="54">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="415" spans="1:6">
+      <c r="A415">
+        <v>202625</v>
+      </c>
+      <c r="B415" s="56">
+        <v>30002114</v>
+      </c>
+      <c r="C415" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D415" s="5">
+        <v>1.135</v>
+      </c>
+      <c r="E415" t="s">
+        <v>484</v>
+      </c>
+      <c r="F415" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="416" spans="1:6">
+      <c r="A416">
+        <v>202625</v>
+      </c>
+      <c r="B416" s="56">
+        <v>30001741</v>
+      </c>
+      <c r="C416" s="5" t="s">
+        <v>508</v>
+      </c>
+      <c r="D416" s="5">
+        <v>1.1152</v>
+      </c>
+      <c r="E416" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="417" spans="1:6">
+      <c r="A417">
+        <v>202625</v>
+      </c>
+      <c r="B417" s="56">
+        <v>30002113</v>
+      </c>
+      <c r="C417" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D417" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="E417" t="s">
+        <v>484</v>
+      </c>
+      <c r="F417" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="418" spans="1:6">
+      <c r="A418">
+        <v>202625</v>
+      </c>
+      <c r="B418" s="56">
+        <v>30000039</v>
+      </c>
+      <c r="C418" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D418" s="5">
+        <v>1.0212000000000001</v>
+      </c>
+      <c r="E418" t="s">
+        <v>530</v>
+      </c>
+      <c r="F418" s="54">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="419" spans="1:6">
+      <c r="A419">
+        <v>202626</v>
+      </c>
+      <c r="B419" s="56">
+        <v>30000560</v>
+      </c>
+      <c r="C419" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="D419" s="5">
+        <v>8.6576000000000004</v>
+      </c>
+      <c r="E419" t="s">
+        <v>531</v>
+      </c>
+      <c r="F419" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="420" spans="1:6">
+      <c r="A420">
+        <v>202626</v>
+      </c>
+      <c r="B420" s="56">
+        <v>30001689</v>
+      </c>
+      <c r="C420" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D420" s="5">
+        <v>7.6075999999999997</v>
+      </c>
+      <c r="E420" t="s">
+        <v>531</v>
+      </c>
+      <c r="F420" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="421" spans="1:6">
+      <c r="A421">
+        <v>202626</v>
+      </c>
+      <c r="B421" s="56">
+        <v>30001815</v>
+      </c>
+      <c r="C421" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="D421" s="6">
+        <v>6.19</v>
+      </c>
+      <c r="E421" t="s">
+        <v>531</v>
+      </c>
+      <c r="F421" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="422" spans="1:6">
+      <c r="A422">
+        <v>202626</v>
+      </c>
+      <c r="B422" s="56">
+        <v>30001773</v>
+      </c>
+      <c r="C422" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="D422" s="5">
+        <v>6.1325599999999998</v>
+      </c>
+      <c r="E422" t="s">
+        <v>531</v>
+      </c>
+      <c r="F422" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="423" spans="1:6">
+      <c r="A423">
+        <v>202626</v>
+      </c>
+      <c r="B423" s="56">
+        <v>30001901</v>
+      </c>
+      <c r="C423" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D423" s="5">
+        <v>5.5944000000000003</v>
+      </c>
+      <c r="E423" t="s">
+        <v>532</v>
+      </c>
+      <c r="F423" s="52">
+        <v>46574</v>
+      </c>
+    </row>
+    <row r="424" spans="1:6">
+      <c r="A424">
+        <v>202626</v>
+      </c>
+      <c r="B424" s="56">
+        <v>30001041</v>
+      </c>
+      <c r="C424" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="D424" s="5">
+        <v>3.1099199999999998</v>
+      </c>
+      <c r="E424" t="s">
+        <v>172</v>
+      </c>
+      <c r="F424" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="425" spans="1:6">
+      <c r="A425">
+        <v>202626</v>
+      </c>
+      <c r="B425" s="56">
+        <v>30000522</v>
+      </c>
+      <c r="C425" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="D425" s="5">
+        <v>101.532</v>
+      </c>
+    </row>
+    <row r="426" spans="1:6">
+      <c r="A426">
+        <v>202626</v>
+      </c>
+      <c r="B426" s="56">
+        <v>30001409</v>
+      </c>
+      <c r="C426" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="D426" s="5">
+        <v>13.497999999999999</v>
+      </c>
+    </row>
+    <row r="427" spans="1:6">
+      <c r="A427">
+        <v>202626</v>
+      </c>
+      <c r="B427" s="56">
+        <v>30001376</v>
+      </c>
+      <c r="C427" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D427" s="5">
+        <v>7.101</v>
+      </c>
+    </row>
+    <row r="428" spans="1:6">
+      <c r="A428">
+        <v>202626</v>
+      </c>
+      <c r="B428" s="56">
+        <v>30001715</v>
+      </c>
+      <c r="C428" s="5" t="s">
+        <v>533</v>
+      </c>
+      <c r="D428" s="5">
+        <v>4.6208</v>
+      </c>
+    </row>
+    <row r="429" spans="1:6">
+      <c r="A429">
+        <v>202626</v>
+      </c>
+      <c r="B429" s="56">
+        <v>30001404</v>
+      </c>
+      <c r="C429" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D429" s="5">
+        <v>4.1085000000000003</v>
+      </c>
+    </row>
+    <row r="430" spans="1:6">
+      <c r="A430">
+        <v>202626</v>
+      </c>
+      <c r="B430" s="56">
+        <v>30001407</v>
+      </c>
+      <c r="C430" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="D430" s="5">
+        <v>3.6044999999999998</v>
+      </c>
+    </row>
+    <row r="431" spans="1:6">
+      <c r="A431">
+        <v>202626</v>
+      </c>
+      <c r="B431" s="56">
+        <v>30000179</v>
+      </c>
+      <c r="C431" s="5" t="s">
+        <v>507</v>
+      </c>
+      <c r="D431" s="5">
+        <v>4.0175999999999998</v>
+      </c>
+    </row>
+    <row r="432" spans="1:6">
+      <c r="A432">
+        <v>202626</v>
+      </c>
+      <c r="B432" s="56">
+        <v>30001142</v>
+      </c>
+      <c r="C432" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D432" s="5">
+        <v>2.085</v>
+      </c>
+      <c r="E432" t="s">
+        <v>534</v>
+      </c>
+      <c r="F432" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="433" spans="1:6">
+      <c r="A433">
+        <v>202626</v>
+      </c>
+      <c r="B433" s="56">
+        <v>30002114</v>
+      </c>
+      <c r="C433" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D433" s="5">
+        <v>1.38</v>
+      </c>
+      <c r="E433" t="s">
+        <v>534</v>
+      </c>
+      <c r="F433" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="434" spans="1:6">
+      <c r="A434">
+        <v>202626</v>
+      </c>
+      <c r="B434" s="56">
+        <v>30001143</v>
+      </c>
+      <c r="C434" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="D434" s="5">
+        <v>1.24</v>
+      </c>
+      <c r="E434" t="s">
+        <v>534</v>
+      </c>
+      <c r="F434" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="435" spans="1:6">
+      <c r="A435">
+        <v>202626</v>
+      </c>
+      <c r="B435" s="56">
+        <v>30000046</v>
+      </c>
+      <c r="C435" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="D435" s="5">
+        <v>1.1592</v>
+      </c>
+      <c r="E435" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="436" spans="1:6">
+      <c r="A436">
+        <v>202626</v>
+      </c>
+      <c r="B436" s="56">
+        <v>30001540</v>
+      </c>
+      <c r="C436" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="D436" s="5">
+        <v>0.65664</v>
+      </c>
+      <c r="E436" t="s">
+        <v>536</v>
+      </c>
+      <c r="F436" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="437" spans="1:6">
+      <c r="A437">
+        <v>202627</v>
+      </c>
+      <c r="B437" s="56">
+        <v>30001901</v>
+      </c>
+      <c r="C437" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="D437" s="6">
+        <v>2.8512</v>
+      </c>
+      <c r="E437" t="s">
+        <v>532</v>
+      </c>
+      <c r="F437" s="52">
+        <v>46574</v>
+      </c>
+    </row>
+    <row r="438" spans="1:6">
+      <c r="A438">
+        <v>202627</v>
+      </c>
+      <c r="B438" s="56">
+        <v>30001689</v>
+      </c>
+      <c r="C438" s="5" t="s">
+        <v>448</v>
+      </c>
+      <c r="D438" s="5">
+        <v>2.6467999999999998</v>
+      </c>
+      <c r="E438" t="s">
+        <v>537</v>
+      </c>
+      <c r="F438" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="439" spans="1:6">
+      <c r="A439">
+        <v>202627</v>
+      </c>
+      <c r="B439" s="56">
+        <v>30002184</v>
+      </c>
+      <c r="C439" s="5" t="s">
+        <v>538</v>
+      </c>
+      <c r="D439" s="5">
+        <v>2.2848000000000002</v>
+      </c>
+      <c r="E439" t="s">
+        <v>539</v>
+      </c>
+      <c r="F439" s="52">
+        <v>46574</v>
+      </c>
+    </row>
+    <row r="440" spans="1:6">
+      <c r="A440">
+        <v>202627</v>
+      </c>
+      <c r="B440" s="56">
+        <v>30002135</v>
+      </c>
+      <c r="C440" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="D440" s="5">
+        <v>2.16</v>
+      </c>
+      <c r="E440" t="s">
+        <v>540</v>
+      </c>
+      <c r="F440" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="441" spans="1:6">
+      <c r="A441">
+        <v>202627</v>
+      </c>
+      <c r="B441" s="56">
+        <v>30001815</v>
+      </c>
+      <c r="C441" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="D441" s="5">
+        <v>2.14</v>
+      </c>
+      <c r="E441" t="s">
+        <v>541</v>
+      </c>
+      <c r="F441" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="442" spans="1:6">
+      <c r="A442">
+        <v>202627</v>
+      </c>
+      <c r="B442" s="56">
+        <v>30002200</v>
+      </c>
+      <c r="C442" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="D442" s="5">
+        <v>1.5407999999999999</v>
+      </c>
+      <c r="E442" t="s">
+        <v>543</v>
+      </c>
+      <c r="F442" s="52">
+        <v>46574</v>
+      </c>
+    </row>
+    <row r="443" spans="1:6">
+      <c r="A443">
+        <v>202627</v>
+      </c>
+      <c r="B443" s="56">
+        <v>30001142</v>
+      </c>
+      <c r="C443" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D443" s="5">
+        <v>1.5149999999999999</v>
+      </c>
+      <c r="E443" t="s">
+        <v>534</v>
+      </c>
+      <c r="F443" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="444" spans="1:6">
+      <c r="A444">
+        <v>202627</v>
+      </c>
+      <c r="B444" s="56">
+        <v>30001143</v>
+      </c>
+      <c r="C444" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="D444" s="5">
+        <v>1.05</v>
+      </c>
+      <c r="E444" t="s">
+        <v>534</v>
+      </c>
+      <c r="F444" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="445" spans="1:6">
+      <c r="A445">
+        <v>202627</v>
+      </c>
+      <c r="B445" s="56">
+        <v>30002114</v>
+      </c>
+      <c r="C445" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D445" s="5">
+        <v>0.755</v>
+      </c>
+      <c r="E445" t="s">
+        <v>534</v>
+      </c>
+      <c r="F445" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="446" spans="1:6">
+      <c r="A446">
+        <v>202627</v>
+      </c>
+      <c r="B446" s="56">
+        <v>30000194</v>
+      </c>
+      <c r="C446" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D446" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="E446" t="s">
+        <v>484</v>
+      </c>
+      <c r="F446" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="447" spans="1:6">
+      <c r="A447">
+        <v>202627</v>
+      </c>
+      <c r="B447" s="56">
+        <v>30001364</v>
+      </c>
+      <c r="C447" s="5" t="s">
+        <v>544</v>
+      </c>
+      <c r="D447" s="5">
+        <v>0.42742000000000002</v>
+      </c>
+      <c r="E447" t="s">
+        <v>545</v>
+      </c>
+      <c r="F447" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="448" spans="1:6">
+      <c r="A448">
+        <v>202627</v>
+      </c>
+      <c r="B448" s="56">
+        <v>30000049</v>
+      </c>
+      <c r="C448" s="5" t="s">
+        <v>546</v>
+      </c>
+      <c r="D448" s="5">
+        <v>0.33119999999999999</v>
+      </c>
+      <c r="F448" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="449" spans="1:6">
+      <c r="A449">
+        <v>202627</v>
+      </c>
+      <c r="B449" s="56">
+        <v>30000522</v>
+      </c>
+      <c r="C449" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="D449" s="5">
+        <v>31.224</v>
+      </c>
+      <c r="E449" t="s">
+        <v>255</v>
+      </c>
+      <c r="F449" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="450" spans="1:6">
+      <c r="A450">
+        <v>202627</v>
+      </c>
+      <c r="B450" s="56">
+        <v>30001409</v>
+      </c>
+      <c r="C450" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="D450" s="5">
+        <v>11.866</v>
+      </c>
+      <c r="E450" t="s">
+        <v>421</v>
+      </c>
+      <c r="F450" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="451" spans="1:6">
+      <c r="A451">
+        <v>202627</v>
+      </c>
+      <c r="B451" s="56">
+        <v>30001376</v>
+      </c>
+      <c r="C451" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D451" s="5">
+        <v>4.4595000000000002</v>
+      </c>
+      <c r="E451" t="s">
+        <v>547</v>
+      </c>
+      <c r="F451" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="452" spans="1:6">
+      <c r="A452">
+        <v>202627</v>
+      </c>
+      <c r="B452" s="56">
+        <v>30001405</v>
+      </c>
+      <c r="C452" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="D452" s="5">
+        <v>3.5640000000000001</v>
+      </c>
+      <c r="E452" t="s">
+        <v>255</v>
+      </c>
+      <c r="F452" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="453" spans="1:6">
+      <c r="A453">
+        <v>202627</v>
+      </c>
+      <c r="B453" s="56">
+        <v>30001404</v>
+      </c>
+      <c r="C453" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D453" s="5">
+        <v>3.5550000000000002</v>
+      </c>
+      <c r="E453" t="s">
+        <v>548</v>
+      </c>
+      <c r="F453" s="54">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="454" spans="1:6">
+      <c r="A454">
+        <v>202627</v>
+      </c>
+      <c r="B454" s="56">
+        <v>30002177</v>
+      </c>
+      <c r="C454" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="D454" s="5">
+        <v>2.1896</v>
+      </c>
+      <c r="E454" t="s">
+        <v>147</v>
+      </c>
+      <c r="F454" t="s">
+        <v>85</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F278"/>
@@ -9873,13 +11708,13 @@
         <v>30001864</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="D2" s="42">
         <v>1235</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>501</v>
+        <v>551</v>
       </c>
       <c r="F2" s="51">
         <v>46104</v>
@@ -9893,16 +11728,16 @@
         <v>30000707</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>502</v>
+        <v>552</v>
       </c>
       <c r="D3" s="42">
         <v>1032</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>503</v>
+        <v>553</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>504</v>
+        <v>554</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -9913,16 +11748,16 @@
         <v>30000824</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>505</v>
+        <v>555</v>
       </c>
       <c r="D4" s="42">
         <v>631</v>
       </c>
       <c r="E4" t="s">
-        <v>506</v>
+        <v>556</v>
       </c>
       <c r="F4" t="s">
-        <v>507</v>
+        <v>557</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -9933,13 +11768,13 @@
         <v>30001001</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>508</v>
+        <v>558</v>
       </c>
       <c r="D5" s="42">
         <v>502</v>
       </c>
       <c r="E5" t="s">
-        <v>506</v>
+        <v>556</v>
       </c>
       <c r="F5" s="52">
         <v>46104</v>
@@ -9953,13 +11788,13 @@
         <v>30000885</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>509</v>
+        <v>559</v>
       </c>
       <c r="D6" s="42">
         <v>440</v>
       </c>
       <c r="E6" t="s">
-        <v>510</v>
+        <v>560</v>
       </c>
       <c r="J6" s="4"/>
     </row>
@@ -9971,16 +11806,16 @@
         <v>30000839</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>511</v>
+        <v>561</v>
       </c>
       <c r="D7" s="42">
         <v>439</v>
       </c>
       <c r="E7" t="s">
-        <v>512</v>
+        <v>562</v>
       </c>
       <c r="F7" t="s">
-        <v>513</v>
+        <v>563</v>
       </c>
       <c r="J7" s="4"/>
     </row>
@@ -9992,13 +11827,13 @@
         <v>30000780</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>514</v>
+        <v>564</v>
       </c>
       <c r="D8" s="42">
         <v>431</v>
       </c>
       <c r="E8" t="s">
-        <v>515</v>
+        <v>565</v>
       </c>
       <c r="J8" s="4"/>
     </row>
@@ -10010,16 +11845,16 @@
         <v>30001701</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>516</v>
+        <v>566</v>
       </c>
       <c r="D9" s="42">
         <v>234</v>
       </c>
       <c r="E9" t="s">
-        <v>517</v>
+        <v>567</v>
       </c>
       <c r="F9" t="s">
-        <v>513</v>
+        <v>563</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -10030,7 +11865,7 @@
         <v>30001864</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="D10" s="5">
         <v>776</v>
@@ -10044,7 +11879,7 @@
         <v>30000814</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>518</v>
+        <v>568</v>
       </c>
       <c r="D11" s="5">
         <v>516</v>
@@ -10058,7 +11893,7 @@
         <v>30000867</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>519</v>
+        <v>569</v>
       </c>
       <c r="D12" s="5">
         <v>347</v>
@@ -10072,7 +11907,7 @@
         <v>30000780</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>514</v>
+        <v>564</v>
       </c>
       <c r="D13" s="5">
         <v>318</v>
@@ -10086,7 +11921,7 @@
         <v>30001001</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>508</v>
+        <v>558</v>
       </c>
       <c r="D14" s="5">
         <v>267</v>
@@ -10100,7 +11935,7 @@
         <v>30000979</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>520</v>
+        <v>570</v>
       </c>
       <c r="D15" s="5">
         <v>160</v>
@@ -10114,7 +11949,7 @@
         <v>30001702</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>521</v>
+        <v>571</v>
       </c>
       <c r="D16" s="5">
         <v>102</v>
@@ -10128,7 +11963,7 @@
         <v>30000811</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>522</v>
+        <v>572</v>
       </c>
       <c r="D17" s="5">
         <v>82</v>
@@ -10142,7 +11977,7 @@
         <v>30001864</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="D18" s="5">
         <v>5085</v>
@@ -10156,7 +11991,7 @@
         <v>30000814</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>518</v>
+        <v>568</v>
       </c>
       <c r="D19" s="5">
         <v>2946</v>
@@ -10170,7 +12005,7 @@
         <v>30001001</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>508</v>
+        <v>558</v>
       </c>
       <c r="D20" s="5">
         <v>1869</v>
@@ -10184,7 +12019,7 @@
         <v>30000803</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>523</v>
+        <v>573</v>
       </c>
       <c r="D21" s="5">
         <v>1590</v>
@@ -10198,7 +12033,7 @@
         <v>30000780</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>514</v>
+        <v>564</v>
       </c>
       <c r="D22" s="5">
         <v>1517</v>
@@ -10212,7 +12047,7 @@
         <v>30000824</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>505</v>
+        <v>555</v>
       </c>
       <c r="D23" s="5">
         <v>1171</v>
@@ -10226,7 +12061,7 @@
         <v>30000707</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>502</v>
+        <v>552</v>
       </c>
       <c r="D24" s="5">
         <v>1032</v>
@@ -10240,7 +12075,7 @@
         <v>30000867</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>519</v>
+        <v>569</v>
       </c>
       <c r="D25" s="5">
         <v>1011</v>
@@ -10254,7 +12089,7 @@
         <v>30000983</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>524</v>
+        <v>574</v>
       </c>
       <c r="D26" s="5">
         <v>169</v>
@@ -10269,7 +12104,7 @@
         <v>30000867</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>519</v>
+        <v>569</v>
       </c>
       <c r="D27" s="5">
         <v>92</v>
@@ -10284,7 +12119,7 @@
         <v>30001570</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>525</v>
+        <v>575</v>
       </c>
       <c r="D28" s="5">
         <v>67</v>
@@ -10299,7 +12134,7 @@
         <v>30001866</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>526</v>
+        <v>576</v>
       </c>
       <c r="D29" s="5">
         <v>62</v>
@@ -10314,7 +12149,7 @@
         <v>30002100</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>527</v>
+        <v>577</v>
       </c>
       <c r="D30" s="5">
         <v>56</v>
@@ -10329,7 +12164,7 @@
         <v>30001702</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>521</v>
+        <v>571</v>
       </c>
       <c r="D31" s="5">
         <v>54</v>
@@ -10344,7 +12179,7 @@
         <v>30000712</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>528</v>
+        <v>578</v>
       </c>
       <c r="D32" s="5">
         <v>53</v>
@@ -10359,7 +12194,7 @@
         <v>30001999</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>529</v>
+        <v>579</v>
       </c>
       <c r="D33" s="5">
         <v>50</v>
@@ -11392,7 +13227,7 @@
   <sheetData>
     <row r="2" spans="2:14" s="22" customFormat="1" ht="15.75">
       <c r="B2" s="20" t="s">
-        <v>530</v>
+        <v>580</v>
       </c>
       <c r="C2" s="28" t="s">
         <v>3</v>
@@ -11402,7 +13237,7 @@
       </c>
       <c r="E2" s="21"/>
       <c r="F2" s="20" t="s">
-        <v>530</v>
+        <v>580</v>
       </c>
       <c r="G2" s="28" t="s">
         <v>3</v>
@@ -11426,13 +13261,13 @@
       </c>
       <c r="E3" s="21"/>
       <c r="F3" s="24" t="s">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="G3" s="29">
         <v>1235</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>531</v>
+        <v>581</v>
       </c>
       <c r="L3" s="41"/>
       <c r="M3" s="39"/>
@@ -11449,13 +13284,13 @@
       </c>
       <c r="E4" s="21"/>
       <c r="F4" s="26" t="s">
-        <v>502</v>
+        <v>552</v>
       </c>
       <c r="G4" s="30">
         <v>1032</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>532</v>
+        <v>582</v>
       </c>
       <c r="L4" s="41"/>
       <c r="M4" s="39"/>
@@ -11472,13 +13307,13 @@
       </c>
       <c r="E5" s="21"/>
       <c r="F5" s="24" t="s">
-        <v>505</v>
+        <v>555</v>
       </c>
       <c r="G5" s="29">
         <v>631</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>531</v>
+        <v>581</v>
       </c>
       <c r="L5" s="41"/>
       <c r="M5" s="38"/>
@@ -11493,13 +13328,13 @@
       <c r="D6" s="25"/>
       <c r="E6" s="21"/>
       <c r="F6" s="26" t="s">
-        <v>508</v>
+        <v>558</v>
       </c>
       <c r="G6" s="30">
         <v>502</v>
       </c>
       <c r="H6" s="25" t="s">
-        <v>531</v>
+        <v>581</v>
       </c>
       <c r="L6" s="41"/>
       <c r="M6" s="38"/>
@@ -11516,13 +13351,13 @@
       </c>
       <c r="E7" s="21"/>
       <c r="F7" s="24" t="s">
-        <v>509</v>
+        <v>559</v>
       </c>
       <c r="G7" s="29">
         <v>440</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>533</v>
+        <v>583</v>
       </c>
       <c r="L7" s="41"/>
       <c r="M7" s="38"/>
@@ -11539,13 +13374,13 @@
       </c>
       <c r="E8" s="21"/>
       <c r="F8" s="26" t="s">
-        <v>511</v>
+        <v>561</v>
       </c>
       <c r="G8" s="33">
         <v>439</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>531</v>
+        <v>581</v>
       </c>
       <c r="L8" s="41"/>
       <c r="M8" s="38"/>
@@ -11562,13 +13397,13 @@
       </c>
       <c r="E9" s="21"/>
       <c r="F9" s="24" t="s">
-        <v>514</v>
+        <v>564</v>
       </c>
       <c r="G9" s="32">
         <v>431</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>531</v>
+        <v>581</v>
       </c>
       <c r="M9" s="38"/>
     </row>
@@ -11584,13 +13419,13 @@
       </c>
       <c r="E10" s="21"/>
       <c r="F10" s="36" t="s">
-        <v>516</v>
+        <v>566</v>
       </c>
       <c r="G10" s="37">
         <v>234</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>531</v>
+        <v>581</v>
       </c>
       <c r="M10" s="38"/>
     </row>

</xml_diff>

<commit_message>
Actualiza reporte S28 (13-Jul-2026) con nuevo archivo WMS
- Adapta carga de stock: nuevo formato DETALLE WMS (antes Stock País agregado)
- Mapea BODEGA WMS → Planta Genérica; agrega stock por SKU total país
- Convierte FCST (toneladas exactitud) a kg para calcular Alcance correctamente
- Normaliza columna "Quebrrados" → "Quebrados" (cambio en Excel)
- S28: Q=246.3t, 107 críticos, 117 alertas

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exactitud-semanal/Principales_Productos_con_Quiebres.xlsx
+++ b/exactitud-semanal/Principales_Productos_con_Quiebres.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1348" uniqueCount="584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1395" uniqueCount="602">
   <si>
     <t xml:space="preserve">Semana </t>
   </si>
@@ -1686,6 +1686,60 @@
   </si>
   <si>
     <t>MANJAR LONCOLECHE BOLSA 10X920GR</t>
+  </si>
+  <si>
+    <t>YOGURT CALAN FTLLA NVA BOL 12X1KG</t>
+  </si>
+  <si>
+    <t>Desvio de junaeb /  13 lunes liberan 20 tons</t>
+  </si>
+  <si>
+    <t>Desvío de demanda / 8 tons</t>
+  </si>
+  <si>
+    <t>Desvío de demanda / poco stock diponible / 8 tons</t>
+  </si>
+  <si>
+    <t>YOGURT CALAN DSCO NVA BOL 12X1KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empalme </t>
+  </si>
+  <si>
+    <t>Falta de material de envase</t>
+  </si>
+  <si>
+    <t>deberia recuperar stock la proxima semana</t>
+  </si>
+  <si>
+    <t>NECTAR WATTS DURAZNO 5X10X115ML</t>
+  </si>
+  <si>
+    <t>Son compras calzadas, se espera vender en Julio el SOP a WMT</t>
+  </si>
+  <si>
+    <t>Semana 28 se producen 40 tons</t>
+  </si>
+  <si>
+    <t>Falta de proteina, stock XLIB</t>
+  </si>
+  <si>
+    <t>LECHE LONCO PROTEIN DESCREMADA 30X200ML</t>
+  </si>
+  <si>
+    <t>Semana 29 se producen 20 tons</t>
+  </si>
+  <si>
+    <t>LECHE BON MOMENT DAN MOCACCINO 30X200ML</t>
+  </si>
+  <si>
+    <t>a la espera de resultados de microbiologia 13 tons</t>
+  </si>
+  <si>
+    <t>Bloqueado</t>
+  </si>
+  <si>
+    <t>Llegada de ME, plan productivo proximas semanas</t>
   </si>
   <si>
     <t>PASTA CHOCLO 12X500GR</t>
@@ -2449,7 +2503,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2558,6 +2612,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
@@ -2880,7 +2935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L454"/>
+  <dimension ref="A1:L489"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="22.85546875" customWidth="1"/>
@@ -9687,10 +9742,10 @@
       <c r="D353" s="58">
         <v>6.9989999999999997</v>
       </c>
-      <c r="E353" s="60" t="s">
+      <c r="E353" s="61" t="s">
         <v>484</v>
       </c>
-      <c r="F353" s="60"/>
+      <c r="F353" s="61"/>
     </row>
     <row r="354" spans="1:7">
       <c r="A354">
@@ -11658,6 +11713,417 @@
       <c r="F454" t="s">
         <v>85</v>
       </c>
+    </row>
+    <row r="455" spans="1:6">
+      <c r="A455">
+        <v>202628</v>
+      </c>
+      <c r="B455" s="60">
+        <v>30001051</v>
+      </c>
+      <c r="C455" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="D455" s="5">
+        <v>15.372</v>
+      </c>
+      <c r="E455" t="s">
+        <v>551</v>
+      </c>
+      <c r="F455" s="54">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="456" spans="1:6">
+      <c r="A456">
+        <v>202628</v>
+      </c>
+      <c r="B456" s="60">
+        <v>30001815</v>
+      </c>
+      <c r="C456" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="D456" s="5">
+        <v>7.21</v>
+      </c>
+      <c r="E456" t="s">
+        <v>552</v>
+      </c>
+      <c r="F456" s="54">
+        <v>46215</v>
+      </c>
+    </row>
+    <row r="457" spans="1:6">
+      <c r="A457">
+        <v>202628</v>
+      </c>
+      <c r="B457" s="60">
+        <v>30000560</v>
+      </c>
+      <c r="C457" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="D457" s="5">
+        <v>4.2279999999999998</v>
+      </c>
+      <c r="E457" t="s">
+        <v>553</v>
+      </c>
+      <c r="F457" s="52">
+        <v>46228</v>
+      </c>
+    </row>
+    <row r="458" spans="1:6">
+      <c r="A458">
+        <v>202628</v>
+      </c>
+      <c r="B458" s="60">
+        <v>30001050</v>
+      </c>
+      <c r="C458" s="5" t="s">
+        <v>554</v>
+      </c>
+      <c r="D458" s="5">
+        <v>3.84</v>
+      </c>
+      <c r="E458" t="s">
+        <v>555</v>
+      </c>
+      <c r="F458" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="459" spans="1:6">
+      <c r="A459">
+        <v>202628</v>
+      </c>
+      <c r="B459" s="60">
+        <v>30001939</v>
+      </c>
+      <c r="C459" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D459" s="5">
+        <v>3.2351999999999999</v>
+      </c>
+      <c r="E459" t="s">
+        <v>555</v>
+      </c>
+      <c r="F459" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="460" spans="1:6">
+      <c r="A460">
+        <v>202628</v>
+      </c>
+      <c r="B460" s="60">
+        <v>30002169</v>
+      </c>
+      <c r="C460" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D460" s="5">
+        <v>2.7378</v>
+      </c>
+      <c r="E460" t="s">
+        <v>556</v>
+      </c>
+      <c r="F460" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="461" spans="1:6">
+      <c r="A461">
+        <v>202628</v>
+      </c>
+      <c r="B461" s="60">
+        <v>30002229</v>
+      </c>
+      <c r="C461" s="5" t="s">
+        <v>558</v>
+      </c>
+      <c r="D461" s="5">
+        <v>15.22025</v>
+      </c>
+      <c r="E461" t="s">
+        <v>559</v>
+      </c>
+      <c r="F461" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="462" spans="1:6">
+      <c r="A462">
+        <v>202628</v>
+      </c>
+      <c r="B462" s="60">
+        <v>30001404</v>
+      </c>
+      <c r="C462" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D462" s="5">
+        <v>10.246499999999999</v>
+      </c>
+      <c r="E462" t="s">
+        <v>560</v>
+      </c>
+      <c r="F462" s="54">
+        <v>46189</v>
+      </c>
+    </row>
+    <row r="463" spans="1:6">
+      <c r="A463">
+        <v>202628</v>
+      </c>
+      <c r="B463" s="60">
+        <v>30001376</v>
+      </c>
+      <c r="C463" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D463" s="5">
+        <v>6.9165000000000001</v>
+      </c>
+      <c r="E463" t="s">
+        <v>561</v>
+      </c>
+      <c r="F463" s="54">
+        <v>46187</v>
+      </c>
+    </row>
+    <row r="464" spans="1:6">
+      <c r="A464">
+        <v>202628</v>
+      </c>
+      <c r="B464" s="60">
+        <v>30002272</v>
+      </c>
+      <c r="C464" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D464" s="5">
+        <v>6.4260000000000002</v>
+      </c>
+      <c r="E464" t="s">
+        <v>563</v>
+      </c>
+      <c r="F464" s="54">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="465" spans="1:6">
+      <c r="A465">
+        <v>202628</v>
+      </c>
+      <c r="B465" s="60">
+        <v>30002177</v>
+      </c>
+      <c r="C465" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="D465" s="5">
+        <v>3.5144000000000002</v>
+      </c>
+      <c r="E465" t="s">
+        <v>421</v>
+      </c>
+      <c r="F465" s="54">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="466" spans="1:6">
+      <c r="A466">
+        <v>202628</v>
+      </c>
+      <c r="B466" s="60">
+        <v>30002358</v>
+      </c>
+      <c r="C466" s="5" t="s">
+        <v>564</v>
+      </c>
+      <c r="D466" s="5">
+        <v>3.012</v>
+      </c>
+      <c r="E466" t="s">
+        <v>565</v>
+      </c>
+      <c r="F466" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="467" spans="1:6">
+      <c r="A467">
+        <v>202628</v>
+      </c>
+      <c r="B467" s="60">
+        <v>30000194</v>
+      </c>
+      <c r="C467" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D467" s="5">
+        <v>3.9089999999999998</v>
+      </c>
+      <c r="E467" t="s">
+        <v>484</v>
+      </c>
+      <c r="F467" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="468" spans="1:6">
+      <c r="A468">
+        <v>202628</v>
+      </c>
+      <c r="B468" s="60">
+        <v>30001143</v>
+      </c>
+      <c r="C468" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="D468" s="5">
+        <v>3.3149999999999999</v>
+      </c>
+      <c r="E468" t="s">
+        <v>567</v>
+      </c>
+      <c r="F468" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="469" spans="1:6">
+      <c r="A469">
+        <v>202628</v>
+      </c>
+      <c r="B469" s="60">
+        <v>30001142</v>
+      </c>
+      <c r="C469" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D469" s="5">
+        <v>3.07</v>
+      </c>
+      <c r="E469" t="s">
+        <v>567</v>
+      </c>
+      <c r="F469" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="470" spans="1:6">
+      <c r="A470">
+        <v>202628</v>
+      </c>
+      <c r="B470" s="60">
+        <v>30000192</v>
+      </c>
+      <c r="C470" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D470" s="5">
+        <v>2.3460000000000001</v>
+      </c>
+      <c r="E470" t="s">
+        <v>255</v>
+      </c>
+      <c r="F470" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="471" spans="1:6">
+      <c r="A471">
+        <v>202628</v>
+      </c>
+      <c r="B471" s="60">
+        <v>30002113</v>
+      </c>
+      <c r="C471" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D471" s="5">
+        <v>2.1800000000000002</v>
+      </c>
+      <c r="E471" t="s">
+        <v>567</v>
+      </c>
+      <c r="F471" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="472" spans="1:6">
+      <c r="A472">
+        <v>202628</v>
+      </c>
+      <c r="B472" s="60">
+        <v>30001698</v>
+      </c>
+      <c r="C472" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="D472" s="5">
+        <v>1.2052799999999999</v>
+      </c>
+      <c r="E472" t="s">
+        <v>534</v>
+      </c>
+      <c r="F472" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="473" spans="1:6">
+      <c r="C473" s="5"/>
+    </row>
+    <row r="474" spans="1:6">
+      <c r="C474" s="5"/>
+    </row>
+    <row r="475" spans="1:6">
+      <c r="C475" s="5"/>
+    </row>
+    <row r="476" spans="1:6">
+      <c r="C476" s="5"/>
+    </row>
+    <row r="477" spans="1:6">
+      <c r="C477" s="5"/>
+    </row>
+    <row r="478" spans="1:6">
+      <c r="C478" s="5"/>
+    </row>
+    <row r="479" spans="1:6">
+      <c r="C479" s="5"/>
+    </row>
+    <row r="480" spans="1:6">
+      <c r="C480" s="5"/>
+    </row>
+    <row r="481" spans="3:3">
+      <c r="C481" s="5"/>
+    </row>
+    <row r="482" spans="3:3">
+      <c r="C482" s="5"/>
+    </row>
+    <row r="483" spans="3:3">
+      <c r="C483" s="5"/>
+    </row>
+    <row r="484" spans="3:3">
+      <c r="C484" s="5"/>
+    </row>
+    <row r="485" spans="3:3">
+      <c r="C485" s="5"/>
+    </row>
+    <row r="486" spans="3:3">
+      <c r="C486" s="5"/>
+    </row>
+    <row r="487" spans="3:3">
+      <c r="C487" s="5"/>
+    </row>
+    <row r="488" spans="3:3">
+      <c r="C488" s="5"/>
+    </row>
+    <row r="489" spans="3:3">
+      <c r="C489" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F278"/>
@@ -11708,13 +12174,13 @@
         <v>30001864</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>550</v>
+        <v>568</v>
       </c>
       <c r="D2" s="42">
         <v>1235</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>551</v>
+        <v>569</v>
       </c>
       <c r="F2" s="51">
         <v>46104</v>
@@ -11728,16 +12194,16 @@
         <v>30000707</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
       <c r="D3" s="42">
         <v>1032</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>553</v>
+        <v>571</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>554</v>
+        <v>572</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -11748,16 +12214,16 @@
         <v>30000824</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>555</v>
+        <v>573</v>
       </c>
       <c r="D4" s="42">
         <v>631</v>
       </c>
       <c r="E4" t="s">
-        <v>556</v>
+        <v>574</v>
       </c>
       <c r="F4" t="s">
-        <v>557</v>
+        <v>575</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -11768,13 +12234,13 @@
         <v>30001001</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>558</v>
+        <v>576</v>
       </c>
       <c r="D5" s="42">
         <v>502</v>
       </c>
       <c r="E5" t="s">
-        <v>556</v>
+        <v>574</v>
       </c>
       <c r="F5" s="52">
         <v>46104</v>
@@ -11788,13 +12254,13 @@
         <v>30000885</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>559</v>
+        <v>577</v>
       </c>
       <c r="D6" s="42">
         <v>440</v>
       </c>
       <c r="E6" t="s">
-        <v>560</v>
+        <v>578</v>
       </c>
       <c r="J6" s="4"/>
     </row>
@@ -11806,16 +12272,16 @@
         <v>30000839</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>561</v>
+        <v>579</v>
       </c>
       <c r="D7" s="42">
         <v>439</v>
       </c>
       <c r="E7" t="s">
-        <v>562</v>
+        <v>580</v>
       </c>
       <c r="F7" t="s">
-        <v>563</v>
+        <v>581</v>
       </c>
       <c r="J7" s="4"/>
     </row>
@@ -11827,13 +12293,13 @@
         <v>30000780</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>564</v>
+        <v>582</v>
       </c>
       <c r="D8" s="42">
         <v>431</v>
       </c>
       <c r="E8" t="s">
-        <v>565</v>
+        <v>583</v>
       </c>
       <c r="J8" s="4"/>
     </row>
@@ -11845,16 +12311,16 @@
         <v>30001701</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>566</v>
+        <v>584</v>
       </c>
       <c r="D9" s="42">
         <v>234</v>
       </c>
       <c r="E9" t="s">
-        <v>567</v>
+        <v>585</v>
       </c>
       <c r="F9" t="s">
-        <v>563</v>
+        <v>581</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -11865,7 +12331,7 @@
         <v>30001864</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>550</v>
+        <v>568</v>
       </c>
       <c r="D10" s="5">
         <v>776</v>
@@ -11879,7 +12345,7 @@
         <v>30000814</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="D11" s="5">
         <v>516</v>
@@ -11893,7 +12359,7 @@
         <v>30000867</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
       <c r="D12" s="5">
         <v>347</v>
@@ -11907,7 +12373,7 @@
         <v>30000780</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>564</v>
+        <v>582</v>
       </c>
       <c r="D13" s="5">
         <v>318</v>
@@ -11921,7 +12387,7 @@
         <v>30001001</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>558</v>
+        <v>576</v>
       </c>
       <c r="D14" s="5">
         <v>267</v>
@@ -11935,7 +12401,7 @@
         <v>30000979</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>570</v>
+        <v>588</v>
       </c>
       <c r="D15" s="5">
         <v>160</v>
@@ -11949,7 +12415,7 @@
         <v>30001702</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>571</v>
+        <v>589</v>
       </c>
       <c r="D16" s="5">
         <v>102</v>
@@ -11963,7 +12429,7 @@
         <v>30000811</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>572</v>
+        <v>590</v>
       </c>
       <c r="D17" s="5">
         <v>82</v>
@@ -11977,7 +12443,7 @@
         <v>30001864</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>550</v>
+        <v>568</v>
       </c>
       <c r="D18" s="5">
         <v>5085</v>
@@ -11991,7 +12457,7 @@
         <v>30000814</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="D19" s="5">
         <v>2946</v>
@@ -12005,7 +12471,7 @@
         <v>30001001</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>558</v>
+        <v>576</v>
       </c>
       <c r="D20" s="5">
         <v>1869</v>
@@ -12019,7 +12485,7 @@
         <v>30000803</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>573</v>
+        <v>591</v>
       </c>
       <c r="D21" s="5">
         <v>1590</v>
@@ -12033,7 +12499,7 @@
         <v>30000780</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>564</v>
+        <v>582</v>
       </c>
       <c r="D22" s="5">
         <v>1517</v>
@@ -12047,7 +12513,7 @@
         <v>30000824</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>555</v>
+        <v>573</v>
       </c>
       <c r="D23" s="5">
         <v>1171</v>
@@ -12061,7 +12527,7 @@
         <v>30000707</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
       <c r="D24" s="5">
         <v>1032</v>
@@ -12075,7 +12541,7 @@
         <v>30000867</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
       <c r="D25" s="5">
         <v>1011</v>
@@ -12089,7 +12555,7 @@
         <v>30000983</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>574</v>
+        <v>592</v>
       </c>
       <c r="D26" s="5">
         <v>169</v>
@@ -12104,7 +12570,7 @@
         <v>30000867</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>569</v>
+        <v>587</v>
       </c>
       <c r="D27" s="5">
         <v>92</v>
@@ -12119,7 +12585,7 @@
         <v>30001570</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>575</v>
+        <v>593</v>
       </c>
       <c r="D28" s="5">
         <v>67</v>
@@ -12134,7 +12600,7 @@
         <v>30001866</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>576</v>
+        <v>594</v>
       </c>
       <c r="D29" s="5">
         <v>62</v>
@@ -12149,7 +12615,7 @@
         <v>30002100</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>577</v>
+        <v>595</v>
       </c>
       <c r="D30" s="5">
         <v>56</v>
@@ -12164,7 +12630,7 @@
         <v>30001702</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>571</v>
+        <v>589</v>
       </c>
       <c r="D31" s="5">
         <v>54</v>
@@ -12179,7 +12645,7 @@
         <v>30000712</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>578</v>
+        <v>596</v>
       </c>
       <c r="D32" s="5">
         <v>53</v>
@@ -12194,7 +12660,7 @@
         <v>30001999</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>579</v>
+        <v>597</v>
       </c>
       <c r="D33" s="5">
         <v>50</v>
@@ -13227,7 +13693,7 @@
   <sheetData>
     <row r="2" spans="2:14" s="22" customFormat="1" ht="15.75">
       <c r="B2" s="20" t="s">
-        <v>580</v>
+        <v>598</v>
       </c>
       <c r="C2" s="28" t="s">
         <v>3</v>
@@ -13237,7 +13703,7 @@
       </c>
       <c r="E2" s="21"/>
       <c r="F2" s="20" t="s">
-        <v>580</v>
+        <v>598</v>
       </c>
       <c r="G2" s="28" t="s">
         <v>3</v>
@@ -13261,13 +13727,13 @@
       </c>
       <c r="E3" s="21"/>
       <c r="F3" s="24" t="s">
-        <v>550</v>
+        <v>568</v>
       </c>
       <c r="G3" s="29">
         <v>1235</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="L3" s="41"/>
       <c r="M3" s="39"/>
@@ -13284,13 +13750,13 @@
       </c>
       <c r="E4" s="21"/>
       <c r="F4" s="26" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
       <c r="G4" s="30">
         <v>1032</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>582</v>
+        <v>600</v>
       </c>
       <c r="L4" s="41"/>
       <c r="M4" s="39"/>
@@ -13307,13 +13773,13 @@
       </c>
       <c r="E5" s="21"/>
       <c r="F5" s="24" t="s">
-        <v>555</v>
+        <v>573</v>
       </c>
       <c r="G5" s="29">
         <v>631</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="L5" s="41"/>
       <c r="M5" s="38"/>
@@ -13328,13 +13794,13 @@
       <c r="D6" s="25"/>
       <c r="E6" s="21"/>
       <c r="F6" s="26" t="s">
-        <v>558</v>
+        <v>576</v>
       </c>
       <c r="G6" s="30">
         <v>502</v>
       </c>
       <c r="H6" s="25" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="L6" s="41"/>
       <c r="M6" s="38"/>
@@ -13351,13 +13817,13 @@
       </c>
       <c r="E7" s="21"/>
       <c r="F7" s="24" t="s">
-        <v>559</v>
+        <v>577</v>
       </c>
       <c r="G7" s="29">
         <v>440</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>583</v>
+        <v>601</v>
       </c>
       <c r="L7" s="41"/>
       <c r="M7" s="38"/>
@@ -13374,13 +13840,13 @@
       </c>
       <c r="E8" s="21"/>
       <c r="F8" s="26" t="s">
-        <v>561</v>
+        <v>579</v>
       </c>
       <c r="G8" s="33">
         <v>439</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="L8" s="41"/>
       <c r="M8" s="38"/>
@@ -13397,13 +13863,13 @@
       </c>
       <c r="E9" s="21"/>
       <c r="F9" s="24" t="s">
-        <v>564</v>
+        <v>582</v>
       </c>
       <c r="G9" s="32">
         <v>431</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="M9" s="38"/>
     </row>
@@ -13419,13 +13885,13 @@
       </c>
       <c r="E10" s="21"/>
       <c r="F10" s="36" t="s">
-        <v>566</v>
+        <v>584</v>
       </c>
       <c r="G10" s="37">
         <v>234</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>581</v>
+        <v>599</v>
       </c>
       <c r="M10" s="38"/>
     </row>

</xml_diff>

<commit_message>
Actualiza datos S28 al 23-Jul-2026
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exactitud-semanal/Principales_Productos_con_Quiebres.xlsx
+++ b/exactitud-semanal/Principales_Productos_con_Quiebres.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1395" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1453" uniqueCount="619">
   <si>
     <t xml:space="preserve">Semana </t>
   </si>
@@ -1740,6 +1740,57 @@
   </si>
   <si>
     <t>Llegada de ME, plan productivo proximas semanas</t>
+  </si>
+  <si>
+    <t>Desvio de demanda (junaeb)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stock disponible </t>
+  </si>
+  <si>
+    <t>YOGURT GRIEGO OIKOS TRZ FRUTILLA 48X110G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desvio de demanda / libera 23 tons el 23 </t>
+  </si>
+  <si>
+    <t>YOGURT GRIEGO OIKOS NAT END 48X110GR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">desvio de ventas </t>
+  </si>
+  <si>
+    <t>falta de material</t>
+  </si>
+  <si>
+    <t>mal cargado fcst de walamart</t>
+  </si>
+  <si>
+    <t>Se retoma para Plan de agosto</t>
+  </si>
+  <si>
+    <t>LECHE LONCO SEMI S/LACTOSA 5X6X200ML</t>
+  </si>
+  <si>
+    <t>Desvío de demanda por mayor catalogacion</t>
+  </si>
+  <si>
+    <t>LECHE FRUTILLA LONCOLECHE 12X1LT</t>
+  </si>
+  <si>
+    <t>Desvío demanda JNB/Dobló su SOP</t>
+  </si>
+  <si>
+    <t>Sin fecha exacta, planes productivos próximas semanas</t>
+  </si>
+  <si>
+    <t>Poca rotación</t>
+  </si>
+  <si>
+    <t>Retraso llegada de ME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin fecha exacta </t>
   </si>
   <si>
     <t>PASTA CHOCLO 12X500GR</t>
@@ -2935,7 +2986,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L489"/>
+  <dimension ref="A1:L493"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="22.85546875" customWidth="1"/>
@@ -12075,55 +12126,421 @@
       </c>
     </row>
     <row r="473" spans="1:6">
-      <c r="C473" s="5"/>
+      <c r="A473">
+        <v>202629</v>
+      </c>
+      <c r="B473" s="56">
+        <v>30001050</v>
+      </c>
+      <c r="C473" s="5" t="s">
+        <v>554</v>
+      </c>
+      <c r="D473" s="5">
+        <v>14.784000000000001</v>
+      </c>
+      <c r="E473" t="s">
+        <v>568</v>
+      </c>
+      <c r="F473" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="474" spans="1:6">
-      <c r="C474" s="5"/>
+      <c r="A474">
+        <v>202629</v>
+      </c>
+      <c r="B474" s="56">
+        <v>30001081</v>
+      </c>
+      <c r="C474" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="D474" s="5">
+        <v>8.6539199999999994</v>
+      </c>
+      <c r="E474" t="s">
+        <v>571</v>
+      </c>
+      <c r="F474" s="54">
+        <v>46226</v>
+      </c>
     </row>
     <row r="475" spans="1:6">
-      <c r="C475" s="5"/>
+      <c r="A475">
+        <v>202629</v>
+      </c>
+      <c r="B475" s="56">
+        <v>30001074</v>
+      </c>
+      <c r="C475" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="D475" s="5">
+        <v>8.5007999999999999</v>
+      </c>
+      <c r="E475" t="s">
+        <v>573</v>
+      </c>
+      <c r="F475" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="476" spans="1:6">
-      <c r="C476" s="5"/>
+      <c r="A476">
+        <v>202629</v>
+      </c>
+      <c r="B476" s="56">
+        <v>30000560</v>
+      </c>
+      <c r="C476" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="D476" s="5">
+        <v>7.4256000000000002</v>
+      </c>
+      <c r="E476" t="s">
+        <v>573</v>
+      </c>
+      <c r="F476" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="477" spans="1:6">
-      <c r="C477" s="5"/>
+      <c r="A477">
+        <v>202629</v>
+      </c>
+      <c r="B477" s="56">
+        <v>30001402</v>
+      </c>
+      <c r="C477" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="D477" s="5">
+        <v>6.3395999999999999</v>
+      </c>
+      <c r="E477" t="s">
+        <v>573</v>
+      </c>
+      <c r="F477" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="478" spans="1:6">
-      <c r="C478" s="5"/>
+      <c r="A478">
+        <v>202629</v>
+      </c>
+      <c r="B478" s="56">
+        <v>30002169</v>
+      </c>
+      <c r="C478" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="D478" s="5">
+        <v>5.0111999999999997</v>
+      </c>
+      <c r="E478" t="s">
+        <v>574</v>
+      </c>
+      <c r="F478" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="479" spans="1:6">
-      <c r="C479" s="5"/>
+      <c r="A479">
+        <v>202629</v>
+      </c>
+      <c r="B479" s="56">
+        <v>30002253</v>
+      </c>
+      <c r="C479" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D479" s="5">
+        <v>4.6818</v>
+      </c>
+      <c r="E479" t="s">
+        <v>575</v>
+      </c>
     </row>
     <row r="480" spans="1:6">
-      <c r="C480" s="5"/>
-    </row>
-    <row r="481" spans="3:3">
-      <c r="C481" s="5"/>
-    </row>
-    <row r="482" spans="3:3">
-      <c r="C482" s="5"/>
-    </row>
-    <row r="483" spans="3:3">
-      <c r="C483" s="5"/>
-    </row>
-    <row r="484" spans="3:3">
-      <c r="C484" s="5"/>
-    </row>
-    <row r="485" spans="3:3">
-      <c r="C485" s="5"/>
-    </row>
-    <row r="486" spans="3:3">
-      <c r="C486" s="5"/>
-    </row>
-    <row r="487" spans="3:3">
-      <c r="C487" s="5"/>
-    </row>
-    <row r="488" spans="3:3">
-      <c r="C488" s="5"/>
-    </row>
-    <row r="489" spans="3:3">
-      <c r="C489" s="5"/>
+      <c r="A480">
+        <v>202629</v>
+      </c>
+      <c r="B480" s="56">
+        <v>30002228</v>
+      </c>
+      <c r="C480" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D480" s="5">
+        <v>14.49</v>
+      </c>
+      <c r="E480" t="s">
+        <v>576</v>
+      </c>
+      <c r="F480" s="54">
+        <v>46234</v>
+      </c>
+    </row>
+    <row r="481" spans="1:6">
+      <c r="A481">
+        <v>202629</v>
+      </c>
+      <c r="B481" s="56">
+        <v>30002229</v>
+      </c>
+      <c r="C481" s="5" t="s">
+        <v>558</v>
+      </c>
+      <c r="D481" s="5">
+        <v>11.908250000000001</v>
+      </c>
+      <c r="E481" t="s">
+        <v>576</v>
+      </c>
+      <c r="F481" s="54">
+        <v>46230</v>
+      </c>
+    </row>
+    <row r="482" spans="1:6">
+      <c r="A482">
+        <v>202629</v>
+      </c>
+      <c r="B482" s="56">
+        <v>30001404</v>
+      </c>
+      <c r="C482" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="D482" s="5">
+        <v>10.102499999999999</v>
+      </c>
+      <c r="E482" t="s">
+        <v>255</v>
+      </c>
+      <c r="F482" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="483" spans="1:6">
+      <c r="A483">
+        <v>202629</v>
+      </c>
+      <c r="B483" s="56">
+        <v>30001376</v>
+      </c>
+      <c r="C483" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="D483" s="5">
+        <v>4.6395</v>
+      </c>
+      <c r="E483" t="s">
+        <v>255</v>
+      </c>
+      <c r="F483" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="484" spans="1:6">
+      <c r="A484">
+        <v>202629</v>
+      </c>
+      <c r="B484" s="56">
+        <v>30000354</v>
+      </c>
+      <c r="C484" s="5" t="s">
+        <v>577</v>
+      </c>
+      <c r="D484" s="5">
+        <v>4.17</v>
+      </c>
+      <c r="E484" t="s">
+        <v>578</v>
+      </c>
+      <c r="F484" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="485" spans="1:6">
+      <c r="A485">
+        <v>202629</v>
+      </c>
+      <c r="B485" s="56">
+        <v>30002066</v>
+      </c>
+      <c r="C485" s="5" t="s">
+        <v>579</v>
+      </c>
+      <c r="D485" s="5">
+        <v>4.1040000000000001</v>
+      </c>
+      <c r="E485" t="s">
+        <v>580</v>
+      </c>
+      <c r="F485" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="486" spans="1:6">
+      <c r="A486">
+        <v>202629</v>
+      </c>
+      <c r="B486" s="56">
+        <v>30002272</v>
+      </c>
+      <c r="C486" s="5" t="s">
+        <v>562</v>
+      </c>
+      <c r="D486" s="5">
+        <v>4.008</v>
+      </c>
+      <c r="E486" t="s">
+        <v>582</v>
+      </c>
+      <c r="F486" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="487" spans="1:6">
+      <c r="A487">
+        <v>202629</v>
+      </c>
+      <c r="B487" s="56">
+        <v>30002113</v>
+      </c>
+      <c r="C487" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D487" s="5">
+        <v>6.165</v>
+      </c>
+      <c r="E487" t="s">
+        <v>583</v>
+      </c>
+      <c r="F487" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="488" spans="1:6">
+      <c r="A488">
+        <v>202629</v>
+      </c>
+      <c r="B488" s="56">
+        <v>30001143</v>
+      </c>
+      <c r="C488" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="D488" s="5">
+        <v>5.9649999999999999</v>
+      </c>
+      <c r="E488" t="s">
+        <v>583</v>
+      </c>
+      <c r="F488" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="489" spans="1:6">
+      <c r="A489">
+        <v>202629</v>
+      </c>
+      <c r="B489" s="56">
+        <v>30001142</v>
+      </c>
+      <c r="C489" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D489" s="5">
+        <v>5.2</v>
+      </c>
+      <c r="E489" t="s">
+        <v>583</v>
+      </c>
+      <c r="F489" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="490" spans="1:6">
+      <c r="A490">
+        <v>202629</v>
+      </c>
+      <c r="B490" s="56">
+        <v>30000194</v>
+      </c>
+      <c r="C490" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D490" s="5">
+        <v>3.7829999999999999</v>
+      </c>
+      <c r="E490" t="s">
+        <v>484</v>
+      </c>
+      <c r="F490" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="491" spans="1:6">
+      <c r="A491">
+        <v>202629</v>
+      </c>
+      <c r="B491" s="56">
+        <v>30002138</v>
+      </c>
+      <c r="C491" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="D491" s="5">
+        <v>2.92</v>
+      </c>
+      <c r="E491" t="s">
+        <v>375</v>
+      </c>
+      <c r="F491" s="54">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="492" spans="1:6">
+      <c r="A492">
+        <v>202629</v>
+      </c>
+      <c r="B492" s="56">
+        <v>30000192</v>
+      </c>
+      <c r="C492" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D492" s="5">
+        <v>2.3639999999999999</v>
+      </c>
+      <c r="E492" t="s">
+        <v>255</v>
+      </c>
+      <c r="F492" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="493" spans="1:6">
+      <c r="A493">
+        <v>202629</v>
+      </c>
+      <c r="B493" s="56">
+        <v>30002114</v>
+      </c>
+      <c r="C493" s="5" t="s">
+        <v>487</v>
+      </c>
+      <c r="D493" s="5">
+        <v>0.875</v>
+      </c>
+      <c r="E493" t="s">
+        <v>583</v>
+      </c>
+      <c r="F493" t="s">
+        <v>581</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F278"/>
@@ -12174,13 +12591,13 @@
         <v>30001864</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>568</v>
+        <v>585</v>
       </c>
       <c r="D2" s="42">
         <v>1235</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>569</v>
+        <v>586</v>
       </c>
       <c r="F2" s="51">
         <v>46104</v>
@@ -12194,16 +12611,16 @@
         <v>30000707</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>570</v>
+        <v>587</v>
       </c>
       <c r="D3" s="42">
         <v>1032</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>571</v>
+        <v>588</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>572</v>
+        <v>589</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -12214,16 +12631,16 @@
         <v>30000824</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>573</v>
+        <v>590</v>
       </c>
       <c r="D4" s="42">
         <v>631</v>
       </c>
       <c r="E4" t="s">
-        <v>574</v>
+        <v>591</v>
       </c>
       <c r="F4" t="s">
-        <v>575</v>
+        <v>592</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -12234,13 +12651,13 @@
         <v>30001001</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>576</v>
+        <v>593</v>
       </c>
       <c r="D5" s="42">
         <v>502</v>
       </c>
       <c r="E5" t="s">
-        <v>574</v>
+        <v>591</v>
       </c>
       <c r="F5" s="52">
         <v>46104</v>
@@ -12254,13 +12671,13 @@
         <v>30000885</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>577</v>
+        <v>594</v>
       </c>
       <c r="D6" s="42">
         <v>440</v>
       </c>
       <c r="E6" t="s">
-        <v>578</v>
+        <v>595</v>
       </c>
       <c r="J6" s="4"/>
     </row>
@@ -12272,16 +12689,16 @@
         <v>30000839</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>579</v>
+        <v>596</v>
       </c>
       <c r="D7" s="42">
         <v>439</v>
       </c>
       <c r="E7" t="s">
-        <v>580</v>
+        <v>597</v>
       </c>
       <c r="F7" t="s">
-        <v>581</v>
+        <v>598</v>
       </c>
       <c r="J7" s="4"/>
     </row>
@@ -12293,13 +12710,13 @@
         <v>30000780</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>582</v>
+        <v>599</v>
       </c>
       <c r="D8" s="42">
         <v>431</v>
       </c>
       <c r="E8" t="s">
-        <v>583</v>
+        <v>600</v>
       </c>
       <c r="J8" s="4"/>
     </row>
@@ -12311,16 +12728,16 @@
         <v>30001701</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>584</v>
+        <v>601</v>
       </c>
       <c r="D9" s="42">
         <v>234</v>
       </c>
       <c r="E9" t="s">
-        <v>585</v>
+        <v>602</v>
       </c>
       <c r="F9" t="s">
-        <v>581</v>
+        <v>598</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -12331,7 +12748,7 @@
         <v>30001864</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>568</v>
+        <v>585</v>
       </c>
       <c r="D10" s="5">
         <v>776</v>
@@ -12345,7 +12762,7 @@
         <v>30000814</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>586</v>
+        <v>603</v>
       </c>
       <c r="D11" s="5">
         <v>516</v>
@@ -12359,7 +12776,7 @@
         <v>30000867</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="D12" s="5">
         <v>347</v>
@@ -12373,7 +12790,7 @@
         <v>30000780</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>582</v>
+        <v>599</v>
       </c>
       <c r="D13" s="5">
         <v>318</v>
@@ -12387,7 +12804,7 @@
         <v>30001001</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>576</v>
+        <v>593</v>
       </c>
       <c r="D14" s="5">
         <v>267</v>
@@ -12401,7 +12818,7 @@
         <v>30000979</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>588</v>
+        <v>605</v>
       </c>
       <c r="D15" s="5">
         <v>160</v>
@@ -12415,7 +12832,7 @@
         <v>30001702</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>589</v>
+        <v>606</v>
       </c>
       <c r="D16" s="5">
         <v>102</v>
@@ -12429,7 +12846,7 @@
         <v>30000811</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>590</v>
+        <v>607</v>
       </c>
       <c r="D17" s="5">
         <v>82</v>
@@ -12443,7 +12860,7 @@
         <v>30001864</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>568</v>
+        <v>585</v>
       </c>
       <c r="D18" s="5">
         <v>5085</v>
@@ -12457,7 +12874,7 @@
         <v>30000814</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>586</v>
+        <v>603</v>
       </c>
       <c r="D19" s="5">
         <v>2946</v>
@@ -12471,7 +12888,7 @@
         <v>30001001</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>576</v>
+        <v>593</v>
       </c>
       <c r="D20" s="5">
         <v>1869</v>
@@ -12485,7 +12902,7 @@
         <v>30000803</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>591</v>
+        <v>608</v>
       </c>
       <c r="D21" s="5">
         <v>1590</v>
@@ -12499,7 +12916,7 @@
         <v>30000780</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>582</v>
+        <v>599</v>
       </c>
       <c r="D22" s="5">
         <v>1517</v>
@@ -12513,7 +12930,7 @@
         <v>30000824</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>573</v>
+        <v>590</v>
       </c>
       <c r="D23" s="5">
         <v>1171</v>
@@ -12527,7 +12944,7 @@
         <v>30000707</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>570</v>
+        <v>587</v>
       </c>
       <c r="D24" s="5">
         <v>1032</v>
@@ -12541,7 +12958,7 @@
         <v>30000867</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="D25" s="5">
         <v>1011</v>
@@ -12555,7 +12972,7 @@
         <v>30000983</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>592</v>
+        <v>609</v>
       </c>
       <c r="D26" s="5">
         <v>169</v>
@@ -12570,7 +12987,7 @@
         <v>30000867</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="D27" s="5">
         <v>92</v>
@@ -12585,7 +13002,7 @@
         <v>30001570</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>593</v>
+        <v>610</v>
       </c>
       <c r="D28" s="5">
         <v>67</v>
@@ -12600,7 +13017,7 @@
         <v>30001866</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>594</v>
+        <v>611</v>
       </c>
       <c r="D29" s="5">
         <v>62</v>
@@ -12615,7 +13032,7 @@
         <v>30002100</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="D30" s="5">
         <v>56</v>
@@ -12630,7 +13047,7 @@
         <v>30001702</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>589</v>
+        <v>606</v>
       </c>
       <c r="D31" s="5">
         <v>54</v>
@@ -12645,7 +13062,7 @@
         <v>30000712</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>596</v>
+        <v>613</v>
       </c>
       <c r="D32" s="5">
         <v>53</v>
@@ -12660,7 +13077,7 @@
         <v>30001999</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>597</v>
+        <v>614</v>
       </c>
       <c r="D33" s="5">
         <v>50</v>
@@ -13693,7 +14110,7 @@
   <sheetData>
     <row r="2" spans="2:14" s="22" customFormat="1" ht="15.75">
       <c r="B2" s="20" t="s">
-        <v>598</v>
+        <v>615</v>
       </c>
       <c r="C2" s="28" t="s">
         <v>3</v>
@@ -13703,7 +14120,7 @@
       </c>
       <c r="E2" s="21"/>
       <c r="F2" s="20" t="s">
-        <v>598</v>
+        <v>615</v>
       </c>
       <c r="G2" s="28" t="s">
         <v>3</v>
@@ -13727,13 +14144,13 @@
       </c>
       <c r="E3" s="21"/>
       <c r="F3" s="24" t="s">
-        <v>568</v>
+        <v>585</v>
       </c>
       <c r="G3" s="29">
         <v>1235</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="L3" s="41"/>
       <c r="M3" s="39"/>
@@ -13750,13 +14167,13 @@
       </c>
       <c r="E4" s="21"/>
       <c r="F4" s="26" t="s">
-        <v>570</v>
+        <v>587</v>
       </c>
       <c r="G4" s="30">
         <v>1032</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>600</v>
+        <v>617</v>
       </c>
       <c r="L4" s="41"/>
       <c r="M4" s="39"/>
@@ -13773,13 +14190,13 @@
       </c>
       <c r="E5" s="21"/>
       <c r="F5" s="24" t="s">
-        <v>573</v>
+        <v>590</v>
       </c>
       <c r="G5" s="29">
         <v>631</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="L5" s="41"/>
       <c r="M5" s="38"/>
@@ -13794,13 +14211,13 @@
       <c r="D6" s="25"/>
       <c r="E6" s="21"/>
       <c r="F6" s="26" t="s">
-        <v>576</v>
+        <v>593</v>
       </c>
       <c r="G6" s="30">
         <v>502</v>
       </c>
       <c r="H6" s="25" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="L6" s="41"/>
       <c r="M6" s="38"/>
@@ -13817,13 +14234,13 @@
       </c>
       <c r="E7" s="21"/>
       <c r="F7" s="24" t="s">
-        <v>577</v>
+        <v>594</v>
       </c>
       <c r="G7" s="29">
         <v>440</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>601</v>
+        <v>618</v>
       </c>
       <c r="L7" s="41"/>
       <c r="M7" s="38"/>
@@ -13840,13 +14257,13 @@
       </c>
       <c r="E8" s="21"/>
       <c r="F8" s="26" t="s">
-        <v>579</v>
+        <v>596</v>
       </c>
       <c r="G8" s="33">
         <v>439</v>
       </c>
       <c r="H8" s="25" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="L8" s="41"/>
       <c r="M8" s="38"/>
@@ -13863,13 +14280,13 @@
       </c>
       <c r="E9" s="21"/>
       <c r="F9" s="24" t="s">
-        <v>582</v>
+        <v>599</v>
       </c>
       <c r="G9" s="32">
         <v>431</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="M9" s="38"/>
     </row>
@@ -13885,13 +14302,13 @@
       </c>
       <c r="E10" s="21"/>
       <c r="F10" s="36" t="s">
-        <v>584</v>
+        <v>601</v>
       </c>
       <c r="G10" s="37">
         <v>234</v>
       </c>
       <c r="H10" s="34" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="M10" s="38"/>
     </row>

</xml_diff>